<commit_message>
added all links back to main excel
</commit_message>
<xml_diff>
--- a/data/Links.xlsx
+++ b/data/Links.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="SEBI"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="54">
   <si>
     <t>Companies Act</t>
   </si>
@@ -146,6 +146,18 @@
   </si>
   <si>
     <t>Listed Companies</t>
+  </si>
+  <si>
+    <t>Circular-BSE</t>
+  </si>
+  <si>
+    <t>https://www.bseindia.com/corporates/CirularToListedComp.html</t>
+  </si>
+  <si>
+    <t>Circular-NSE</t>
+  </si>
+  <si>
+    <t>https://www.nseindia.com/companies-listing/circular-for-listed-companies-equity-market</t>
   </si>
   <si>
     <t>SEBI</t>
@@ -631,7 +643,7 @@
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
       <c r="A1" s="7"/>
       <c r="B1" s="8" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
@@ -663,7 +675,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -695,7 +707,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -724,10 +736,10 @@
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
       <c r="A4" s="3" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -759,7 +771,7 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -791,7 +803,7 @@
         <v>24</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -823,7 +835,7 @@
         <v>39</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -28716,8 +28728,12 @@
       <c r="U1" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4"/>
+      <c r="A2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>43</v>
+      </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
@@ -28738,9 +28754,13 @@
       <c r="T2" s="7"/>
       <c r="U2" s="7"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
+      <c r="A3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>45</v>
+      </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
       <c r="E3" s="7"/>
@@ -51833,7 +51853,7 @@
         <v>21</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="31.5">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -51841,7 +51861,7 @@
         <v>22</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="31.5">
       <c r="A3" s="3" t="s">
         <v>5</v>
       </c>
@@ -51849,7 +51869,7 @@
         <v>23</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="31.5">
       <c r="A4" s="3" t="s">
         <v>24</v>
       </c>
@@ -51857,7 +51877,7 @@
         <v>25</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="31.5">
       <c r="A5" s="3" t="s">
         <v>26</v>
       </c>

</xml_diff>